<commit_message>
task-2360: pivot hides the Values row like Excel, error cells stay inline, clippy clean, merge fixes
</commit_message>
<xml_diff>
--- a/crates/unluminous-sheet/_agent_output/pivot/explore/exp1/b6.xlsx
+++ b/crates/unluminous-sheet/_agent_output/pivot/explore/exp1/b6.xlsx
@@ -960,6 +960,11 @@
     <dataField name="Sum of Amount" fld="6" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+  </extLst>
 </pivotTableDefinition>
 </file>
 

</xml_diff>